<commit_message>
feat: implement backend schemas and service logic for QR-based access control and visitor management
</commit_message>
<xml_diff>
--- a/pruebas_pases_10_pax.xlsx
+++ b/pruebas_pases_10_pax.xlsx
@@ -521,52 +521,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MATILDE PI GILABERT</t>
+          <t>FLORINA CARRO</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>E-21008795</t>
+          <t>V-29168748</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>torremaria-manuela@example.net</t>
+          <t>gutierrezprudencio@example.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>04242767391</t>
+          <t>04241154028</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>WTP859</t>
+          <t>SSD-272</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>JEEP</t>
+          <t>RENAULT</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CHEROKEE</t>
+          <t>DUSTER</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>GRIS</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+          <t>PLATA</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>JQH-724</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CHEVROLET</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>OPTRA</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>NFN-709</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>TOYOTA</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>YARIS</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
@@ -575,52 +607,84 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>JAVIER BARRAGÁN ARÉVALO</t>
+          <t>FABRICIO JOSE CARLOS ABAD HERVIA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>V-23780357</t>
+          <t>E-22793804</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>alexandra74@example.org</t>
+          <t>rosellomaximiano@example.net</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>04240575333</t>
+          <t>04243508196</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>KGO-569</t>
+          <t>AC762BA</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>TOYOTA</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>HILUX</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>GRIS</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>AC323BA</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>RENAULT</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>LOGAN</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>PLATA</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>DUSTER</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>BYU-515</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>TOYOTA</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>FORTUNER</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>AZUL</t>
+        </is>
+      </c>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
@@ -629,52 +693,84 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALEJANDRO LOZANO ARIÑO</t>
+          <t>GERTRUDIS VÉLEZ-BARROSO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>E-14848489</t>
+          <t>V-30759175</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nsanchez@example.com</t>
+          <t>uferrero@example.org</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>04144005367</t>
+          <t>02122458936</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>TTG531</t>
+          <t>AC497BA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>MITSUBISHI</t>
+          <t>FORD</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>MONTERO</t>
+          <t>FIESTA</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AC938BA</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>TUCSON</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>VERDE</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>AC778BA</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>RENAULT</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>LOGAN</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>ROJO</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
@@ -683,52 +779,84 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PILI BERENGUER-GARAY</t>
+          <t>JOSEFINA LLADÓ BARBERÁ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>E-29783717</t>
+          <t>E-16314512</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>nieves93@example.com</t>
+          <t>alcazarreinaldo@example.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>04122959152</t>
+          <t>04144492354</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ZQZ-993</t>
+          <t>EJJ-082</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>HYUNDAI</t>
+          <t>CHEVROLET</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>GETZ</t>
+          <t>AVEO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>DCU662</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>JEEP</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>WRANGLER</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>AC120BA</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>RENAULT</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>DUSTER</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>PLATA</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
@@ -737,52 +865,84 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EVARISTO BERNAL ALCÁZAR</t>
+          <t>OFELIA TORMO GALÁN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>V-18463384</t>
+          <t>V-12922947</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>rbayon@example.net</t>
+          <t>fitovera@example.org</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>04140908036</t>
+          <t>04269342780</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FGK-344</t>
+          <t>FYR-946</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>MITSUBISHI</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>MONTERO</t>
+          <t>ELANTRA</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>AZUL</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>AC576BA</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>RENAULT</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>LOGAN</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>XYM-796</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>FORD</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>F-150</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>GRIS</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
@@ -791,27 +951,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FABIOLA SILVA BALAGUER</t>
+          <t>TERE SOLANA MORELL</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>E-9949694</t>
+          <t>V-29153023</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>yjurado@example.net</t>
+          <t>ymercader@example.org</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>02123421568</t>
+          <t>04122783743</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AC371BA</t>
+          <t>AC726BA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -821,22 +981,54 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>WRANGLER</t>
+          <t>CHEROKEE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PLATA</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>NOX789</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>TOYOTA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FORTUNER</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>BOI050</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>TUCSON</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>VERDE</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
@@ -845,52 +1037,84 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EVANGELINA CORBACHO TRUJILLO</t>
+          <t>AARÓN SAMPER PRAT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>V-22606469</t>
+          <t>E-21554749</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>maria-josebenavent@example.com</t>
+          <t>maria-manuelaborja@example.org</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>04263737899</t>
+          <t>02122096141</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AC778BA</t>
+          <t>AC408BA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>JEEP</t>
+          <t>HYUNDAI</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CHEROKEE</t>
+          <t>GETZ</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>AZUL</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+          <t>PLATA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>GRP-947</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>GETZ</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>EZF908</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>CHEVROLET</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>SILVERADO</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>PLATA</t>
+        </is>
+      </c>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
@@ -899,52 +1123,84 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FRANCISCA GALÁN</t>
+          <t>MARTIN ATILIO QUINTANILLA ROMÁN</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>E-10540166</t>
+          <t>V-25925411</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>vfabregas@example.net</t>
+          <t>eustaquioacevedo@example.org</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>02123837879</t>
+          <t>04244629224</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AC838BA</t>
+          <t>AC780BA</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>RENAULT</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>LOGAN</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ULX-437</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>FORD</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FIESTA</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>PLATA</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>AC483BA</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
           <t>HYUNDAI</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>TUCSON</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>AZUL</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>GETZ</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>VERDE</t>
+        </is>
+      </c>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
@@ -953,37 +1209,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LEYRE DIAZ LUZ</t>
+          <t>ELIGIA PORCEL-PONS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>E-9413867</t>
+          <t>V-29022848</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>pfajardo@example.org</t>
+          <t>sol85@example.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>02129121255</t>
+          <t>04120689374</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>OYU271</t>
+          <t>AC678BA</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>JEEP</t>
+          <t>CHEVROLET</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>CHEROKEE</t>
+          <t>OPTRA</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -991,14 +1247,46 @@
           <t>GRIS</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>JOH125</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>RENAULT</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>LOGAN</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>GRIS</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>JGR705</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>HYUNDAI</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>TUCSON</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>GRIS</t>
+        </is>
+      </c>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
@@ -1007,52 +1295,84 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CARLITO ESPAÑOL SOLSONA</t>
+          <t>ALMA MANCEBO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>V-9009664</t>
+          <t>V-10923275</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>msarabia@example.org</t>
+          <t>ppi@example.net</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>04122580453</t>
+          <t>04120059400</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AC342BA</t>
+          <t>POS-668</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>MITSUBISHI</t>
+          <t>JEEP</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MONTERO</t>
+          <t>WRANGLER</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>GRIS</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>AC868BA</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>FORD</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FIESTA</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>VKN003</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>CHEVROLET</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>AVEO</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>BLANCO</t>
+        </is>
+      </c>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: implement PasesMasivos page for bulk pass management and add sample Excel templates for testing.
</commit_message>
<xml_diff>
--- a/pruebas_pases_10_pax.xlsx
+++ b/pruebas_pases_10_pax.xlsx
@@ -521,84 +521,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FLORINA CARRO</t>
+          <t>OLGA MARTÍ BAUZÀ</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>V-29168748</t>
+          <t>V-17948018</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>gutierrezprudencio@example.com</t>
+          <t>valenciaconrado@example.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>04241154028</t>
+          <t>04262092360</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>SSD-272</t>
+          <t>AC406BA</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>RENAULT</t>
+          <t>JEEP</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>DUSTER</t>
+          <t>WRANGLER</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>PLATA</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>JQH-724</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>CHEVROLET</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>OPTRA</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>NEGRO</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>NFN-709</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>TOYOTA</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>YARIS</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>NEGRO</t>
-        </is>
-      </c>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
@@ -607,84 +575,52 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FABRICIO JOSE CARLOS ABAD HERVIA</t>
+          <t>MAXIMIANO CARVAJAL</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>E-22793804</t>
+          <t>V-29505636</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>rosellomaximiano@example.net</t>
+          <t>tporras@example.net</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>04243508196</t>
+          <t>02125008637</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AC762BA</t>
+          <t>LIE-439</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TOYOTA</t>
+          <t>RENAULT</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>HILUX</t>
+          <t>DUSTER</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>GRIS</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>AC323BA</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>RENAULT</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>DUSTER</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>ROJO</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>BYU-515</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>TOYOTA</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>FORTUNER</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>AZUL</t>
-        </is>
-      </c>
+          <t>BLANCO</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
@@ -693,84 +629,52 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GERTRUDIS VÉLEZ-BARROSO</t>
+          <t>JOVITA CORBACHO BARROSO</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>V-30759175</t>
+          <t>V-29185064</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>uferrero@example.org</t>
+          <t>cabelloreynaldo@example.net</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>02122458936</t>
+          <t>02129551668</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>AC497BA</t>
+          <t>AC870BA</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>FORD</t>
+          <t>JEEP</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>FIESTA</t>
+          <t>WRANGLER</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ROJO</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>AC938BA</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>HYUNDAI</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>TUCSON</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>VERDE</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>AC778BA</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>RENAULT</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>LOGAN</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>ROJO</t>
-        </is>
-      </c>
+          <t>GRIS</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
@@ -779,84 +683,52 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JOSEFINA LLADÓ BARBERÁ</t>
+          <t>ADORACIÓN ARAUJO CORREA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>E-16314512</t>
+          <t>E-8114951</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>alcazarreinaldo@example.com</t>
+          <t>angelina66@example.net</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>04144492354</t>
+          <t>04247417460</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>EJJ-082</t>
+          <t>FXF542</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CHEVROLET</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>AVEO</t>
+          <t>YARIS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NEGRO</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>DCU662</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>JEEP</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>WRANGLER</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
           <t>VERDE</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>AC120BA</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>RENAULT</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>DUSTER</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>PLATA</t>
-        </is>
-      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
@@ -865,37 +737,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>OFELIA TORMO GALÁN</t>
+          <t>BALDOMERO VARGAS-SOMOZA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>V-12922947</t>
+          <t>E-29937427</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>fitovera@example.org</t>
+          <t>terronpiedad@example.org</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>04269342780</t>
+          <t>02128393379</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FYR-946</t>
+          <t>AC966BA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>HYUNDAI</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ELANTRA</t>
+          <t>YARIS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -903,46 +775,14 @@
           <t>AZUL</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>AC576BA</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>RENAULT</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>LOGAN</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>NEGRO</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>XYM-796</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>FORD</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>F-150</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>GRIS</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
@@ -951,84 +791,52 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TERE SOLANA MORELL</t>
+          <t>ELISEO PINEDA CASES</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>V-29153023</t>
+          <t>E-26304516</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ymercader@example.org</t>
+          <t>ivan40@example.net</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>04122783743</t>
+          <t>04269697707</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AC726BA</t>
+          <t>AC575BA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>JEEP</t>
+          <t>FORD</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CHEROKEE</t>
+          <t>FIESTA</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>BLANCO</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>NOX789</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>TOYOTA</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>FORTUNER</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>ROJO</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>BOI050</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>HYUNDAI</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>TUCSON</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>VERDE</t>
-        </is>
-      </c>
+          <t>GRIS</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
@@ -1037,84 +845,52 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AARÓN SAMPER PRAT</t>
+          <t>LINA VIDAL-MORANTE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E-21554749</t>
+          <t>V-15673724</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>maria-manuelaborja@example.org</t>
+          <t>lizquierdo@example.net</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>02122096141</t>
+          <t>04142856509</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AC408BA</t>
+          <t>AC497BA</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>HYUNDAI</t>
+          <t>TOYOTA</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>GETZ</t>
+          <t>FORTUNER</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>PLATA</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>GRP-947</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>HYUNDAI</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>GETZ</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>NEGRO</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>EZF908</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>CHEVROLET</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>SILVERADO</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>PLATA</t>
-        </is>
-      </c>
+          <t>VERDE</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
@@ -1123,37 +899,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MARTIN ATILIO QUINTANILLA ROMÁN</t>
+          <t>ELADIO LEÓN LANDA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>V-25925411</t>
+          <t>E-9482719</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>eustaquioacevedo@example.org</t>
+          <t>sosimo24@example.net</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>04244629224</t>
+          <t>04141651544</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AC780BA</t>
+          <t>QBB-326</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>RENAULT</t>
+          <t>JEEP</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>LOGAN</t>
+          <t>CHEROKEE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1161,46 +937,14 @@
           <t>VERDE</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>ULX-437</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>FORD</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>FIESTA</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>PLATA</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>AC483BA</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>HYUNDAI</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>GETZ</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>VERDE</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
@@ -1209,27 +953,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ELIGIA PORCEL-PONS</t>
+          <t>XIOMARA AGUADO-RODRÍGUEZ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>V-29022848</t>
+          <t>E-30556521</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>sol85@example.com</t>
+          <t>ppujol@example.org</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>04120689374</t>
+          <t>04149802188</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AC678BA</t>
+          <t>DGW762</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1244,49 +988,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>GRIS</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>JOH125</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>RENAULT</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>LOGAN</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>GRIS</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>JGR705</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>HYUNDAI</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>TUCSON</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>GRIS</t>
-        </is>
-      </c>
+          <t>NEGRO</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
@@ -1295,84 +1007,52 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ALMA MANCEBO</t>
+          <t>HORTENSIA HAYDÉE PALAU PALMER</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>V-10923275</t>
+          <t>E-12963332</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ppi@example.net</t>
+          <t>cruzsacristan@example.net</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>04120059400</t>
+          <t>02128546174</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>POS-668</t>
+          <t>AC199BA</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>JEEP</t>
+          <t>MITSUBISHI</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>WRANGLER</t>
+          <t>LANCER</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>VERDE</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>AC868BA</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>FORD</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>FIESTA</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>NEGRO</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>VKN003</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>CHEVROLET</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>AVEO</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>BLANCO</t>
-        </is>
-      </c>
+          <t>ROJO</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>

</xml_diff>